<commit_message>
Changed to U235 (thermal fission) decay heat data as this leads to better agreement with reported decay heat fractions. Cleaned up the code.
</commit_message>
<xml_diff>
--- a/pointkinetics/ANS Decay heat data.xlsx
+++ b/pointkinetics/ANS Decay heat data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\poncet_m\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\poncetma\modelica\models\pointkinetics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3261169D-8373-4940-A035-43DEA2F51516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{462489CE-7EC4-44F5-80A8-D1822703C249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12585" xr2:uid="{4E68769E-48B3-45EE-AC69-8947B5286AD2}"/>
+    <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="12585" xr2:uid="{4E68769E-48B3-45EE-AC69-8947B5286AD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
-  <si>
-    <t>1.8531E—07</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t>alpha_i</t>
   </si>
@@ -57,6 +54,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000E+00"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -86,9 +86,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,37 +406,41 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7855CBB7-039F-4013-854C-E58C61D98982}">
   <dimension ref="C2:I26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" t="s">
-        <v>2</v>
-      </c>
       <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
         <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="4" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>0.65056999999999998</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>22.138000000000002</v>
       </c>
       <c r="F4" s="1">
@@ -455,10 +460,10 @@
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>0.51263999999999998</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>0.51587000000000005</v>
       </c>
       <c r="F5" s="1">
@@ -478,10 +483,10 @@
       <c r="C6">
         <v>3</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>0.24384</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>0.19594</v>
       </c>
       <c r="F6" s="1">
@@ -501,10 +506,10 @@
       <c r="C7">
         <v>4</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="2">
         <v>0.13850000000000001</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>0.10314</v>
       </c>
       <c r="F7" s="1">
@@ -524,10 +529,10 @@
       <c r="C8">
         <v>5</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>5.5440000000000003E-2</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>3.3655999999999998E-2</v>
       </c>
       <c r="F8" s="1">
@@ -547,10 +552,10 @@
       <c r="C9">
         <v>6</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="2">
         <v>2.2225000000000002E-2</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>1.1681E-2</v>
       </c>
       <c r="F9" s="1">
@@ -570,10 +575,10 @@
       <c r="C10">
         <v>7</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="2">
         <v>3.3088000000000002E-3</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>3.5869999999999999E-3</v>
       </c>
       <c r="F10" s="1">
@@ -593,10 +598,10 @@
       <c r="C11">
         <v>8</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="2">
         <v>9.3015000000000003E-4</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>1.3929999999999999E-3</v>
       </c>
       <c r="F11" s="1">
@@ -616,10 +621,10 @@
       <c r="C12">
         <v>9</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>8.0942999999999998E-4</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>6.2629999999999999E-4</v>
       </c>
       <c r="F12" s="1">
@@ -639,10 +644,10 @@
       <c r="C13">
         <v>10</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>1.9567E-4</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>1.8906000000000001E-4</v>
       </c>
       <c r="F13" s="1">
@@ -662,10 +667,10 @@
       <c r="C14">
         <v>11</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>3.2534999999999999E-5</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>5.4988000000000003E-5</v>
       </c>
       <c r="F14" s="1">
@@ -685,10 +690,10 @@
       <c r="C15">
         <v>12</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>7.5595000000000002E-6</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>2.0958000000000002E-5</v>
       </c>
       <c r="F15" s="1">
@@ -708,10 +713,10 @@
       <c r="C16">
         <v>13</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>2.5231999999999998E-6</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>1.0010000000000001E-5</v>
       </c>
       <c r="F16" s="1">
@@ -731,10 +736,10 @@
       <c r="C17">
         <v>14</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>4.9948000000000002E-7</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>2.5438000000000001E-6</v>
       </c>
       <c r="F17" s="1">
@@ -754,10 +759,10 @@
       <c r="C18">
         <v>15</v>
       </c>
-      <c r="D18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E18" s="1">
+      <c r="D18" s="2">
+        <v>1.8531000000000001E-7</v>
+      </c>
+      <c r="E18" s="2">
         <v>6.6361000000000005E-7</v>
       </c>
       <c r="F18" s="1">
@@ -777,10 +782,10 @@
       <c r="C19">
         <v>16</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>2.6607999999999999E-8</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>1.229E-7</v>
       </c>
       <c r="F19" s="1">
@@ -800,10 +805,10 @@
       <c r="C20">
         <v>17</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>2.2398000000000001E-9</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>2.7213E-8</v>
       </c>
       <c r="F20" s="1">
@@ -823,10 +828,10 @@
       <c r="C21">
         <v>18</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>8.1641000000000007E-12</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>4.3714E-9</v>
       </c>
       <c r="F21" s="1">
@@ -846,10 +851,10 @@
       <c r="C22">
         <v>19</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>8.7796999999999997E-11</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>7.5780000000000001E-10</v>
       </c>
       <c r="F22" s="1">
@@ -869,10 +874,10 @@
       <c r="C23">
         <v>20</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>2.5130999999999999E-14</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>2.4786000000000001E-10</v>
       </c>
       <c r="F23" s="1">
@@ -892,10 +897,10 @@
       <c r="C24">
         <v>21</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="2">
         <v>3.2175999999999998E-16</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>2.2384000000000001E-13</v>
       </c>
       <c r="F24" s="1">
@@ -915,10 +920,10 @@
       <c r="C25">
         <v>22</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="2">
         <v>4.5037999999999997E-17</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>2.4600000000000001E-14</v>
       </c>
       <c r="F25" s="1">
@@ -938,10 +943,10 @@
       <c r="C26">
         <v>23</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>7.4790999999999996E-17</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>1.5698999999999999E-14</v>
       </c>
       <c r="F26" s="1">
@@ -959,5 +964,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>